<commit_message>
Add User ID column to User excel
</commit_message>
<xml_diff>
--- a/wwwroot/templates/KullaniciTemplate.xlsx
+++ b/wwwroot/templates/KullaniciTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EMutabakat\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{849F1ED3-68BF-4DC0-B70D-689666362169}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96946AA8-8626-44EF-A635-A565AB7AD81C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2625" yWindow="3195" windowWidth="18795" windowHeight="11115" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4440" yWindow="1455" windowWidth="16950" windowHeight="11115" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>FirmaId</t>
   </si>
@@ -44,6 +44,9 @@
   </si>
   <si>
     <t>Rol</t>
+  </si>
+  <si>
+    <t>KullaniciId</t>
   </si>
 </sst>
 </file>
@@ -383,41 +386,45 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.28515625" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" customWidth="1"/>
-    <col min="4" max="4" width="16.85546875" customWidth="1"/>
-    <col min="5" max="5" width="17.85546875" customWidth="1"/>
-    <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="16.5703125" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" customWidth="1"/>
+    <col min="6" max="6" width="17.85546875" customWidth="1"/>
+    <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11" customWidth="1"/>
+    <col min="9" max="9" width="16.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add multi-firma support to User Excel import flow
</commit_message>
<xml_diff>
--- a/wwwroot/templates/KullaniciTemplate.xlsx
+++ b/wwwroot/templates/KullaniciTemplate.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOD\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EMutabakat\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0303EEB-B53E-469E-BD1F-3BD723BBAF13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82315EAB-9F4D-4FB5-AD49-55A6F6A40000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8925" yWindow="8250" windowWidth="16950" windowHeight="11115" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7500" yWindow="4485" windowWidth="16950" windowHeight="11115" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
-  <si>
-    <t>FirmaId</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
   <si>
     <t>KullaniciAdi</t>
   </si>
@@ -428,22 +425,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" customWidth="1"/>
-    <col min="5" max="5" width="16.85546875" customWidth="1"/>
-    <col min="6" max="6" width="17.85546875" customWidth="1"/>
-    <col min="7" max="7" width="16.5703125" customWidth="1"/>
-    <col min="8" max="8" width="17" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" customWidth="1"/>
+    <col min="4" max="4" width="16.85546875" customWidth="1"/>
+    <col min="5" max="5" width="17.85546875" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" customWidth="1"/>
+    <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -458,110 +455,98 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" t="s">
         <v>4</v>
-      </c>
-      <c r="G1" t="s">
-        <v>7</v>
       </c>
       <c r="H1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" t="s">
-        <v>6</v>
-      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2</v>
       </c>
-      <c r="B2">
-        <v>1</v>
+      <c r="B2" t="s">
+        <v>7</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2">
+      <c r="D2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2">
         <v>5551112233</v>
       </c>
-      <c r="G2" t="s">
-        <v>14</v>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
       </c>
       <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="I2">
         <v>111111</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>3</v>
       </c>
-      <c r="B3">
-        <v>1</v>
+      <c r="B3" t="s">
+        <v>10</v>
       </c>
       <c r="C3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3">
+      <c r="D3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3">
         <v>5551112233</v>
       </c>
-      <c r="G3" t="s">
-        <v>10</v>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
       </c>
       <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3">
         <v>111111</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>4</v>
       </c>
-      <c r="B4">
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4">
+        <v>5551112233</v>
+      </c>
+      <c r="F4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4">
         <v>1</v>
       </c>
-      <c r="C4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4">
-        <v>5551112233</v>
-      </c>
-      <c r="G4" t="s">
-        <v>14</v>
-      </c>
       <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4">
         <v>111111</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{9C469817-3926-4F8D-B5ED-8556D44BDE9B}"/>
-    <hyperlink ref="E3" r:id="rId2" xr:uid="{3690221B-13B7-46CD-97F5-2E6760F937F2}"/>
-    <hyperlink ref="E4" r:id="rId3" xr:uid="{799CCEB2-4032-4FB2-AD04-A24C627D1575}"/>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{9C469817-3926-4F8D-B5ED-8556D44BDE9B}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{3690221B-13B7-46CD-97F5-2E6760F937F2}"/>
+    <hyperlink ref="D4" r:id="rId3" xr:uid="{799CCEB2-4032-4FB2-AD04-A24C627D1575}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Implement upsert logic in User Excel import
</commit_message>
<xml_diff>
--- a/wwwroot/templates/KullaniciTemplate.xlsx
+++ b/wwwroot/templates/KullaniciTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EMutabakat\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82315EAB-9F4D-4FB5-AD49-55A6F6A40000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0FA8C63-F6BA-49DD-AC24-667530EA5BAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7500" yWindow="4485" windowWidth="16950" windowHeight="11115" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="990" yWindow="3975" windowWidth="16950" windowHeight="10935" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
@@ -46,9 +46,6 @@
     <t>Kübra</t>
   </si>
   <si>
-    <t>Varol</t>
-  </si>
-  <si>
     <t>Admin</t>
   </si>
   <si>
@@ -77,6 +74,9 @@
   </si>
   <si>
     <t>aysedemir@gmail.com</t>
+  </si>
+  <si>
+    <t>Varoloooo</t>
   </si>
 </sst>
 </file>
@@ -440,7 +440,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -472,16 +472,16 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E2">
         <v>5551112233</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -495,19 +495,19 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
       <c r="D3" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E3">
         <v>5551112233</v>
       </c>
       <c r="F3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -521,19 +521,19 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E4">
         <v>5551112233</v>
       </c>
       <c r="F4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G4">
         <v>1</v>

</xml_diff>

<commit_message>
Renew user excel template with updated one
</commit_message>
<xml_diff>
--- a/wwwroot/templates/KullaniciTemplate.xlsx
+++ b/wwwroot/templates/KullaniciTemplate.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr codeName="ThisWorkbook"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EMutabakat\wwwroot\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOD\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0FA8C63-F6BA-49DD-AC24-667530EA5BAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F117C2D-5886-420E-8AA7-B670E00F72D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="990" yWindow="3975" windowWidth="16950" windowHeight="10935" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="690" yWindow="4275" windowWidth="16950" windowHeight="10950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+  <si>
+    <t>KullaniciId</t>
+  </si>
   <si>
     <t>KullaniciAdi</t>
   </si>
@@ -34,49 +37,49 @@
     <t>KullaniciGsm</t>
   </si>
   <si>
+    <t>Rol</t>
+  </si>
+  <si>
     <t>KullanıcıAktifPasif</t>
   </si>
   <si>
     <t>Sifre</t>
   </si>
   <si>
-    <t>Rol</t>
-  </si>
-  <si>
     <t>Kübra</t>
   </si>
   <si>
+    <t>kubravarol@gmail.com</t>
+  </si>
+  <si>
+    <t>Standart</t>
+  </si>
+  <si>
+    <t>Ahmet</t>
+  </si>
+  <si>
+    <t>Yılmaz</t>
+  </si>
+  <si>
+    <t>ahmetyılmaz@gmail.com</t>
+  </si>
+  <si>
     <t>Admin</t>
   </si>
   <si>
-    <t>Ahmet</t>
-  </si>
-  <si>
-    <t>Yılmaz</t>
-  </si>
-  <si>
     <t>Ayşe</t>
   </si>
   <si>
-    <t>Standart</t>
-  </si>
-  <si>
-    <t>KullaniciId</t>
-  </si>
-  <si>
     <t>Demir</t>
   </si>
   <si>
-    <t>kubravarol@gmail.com</t>
-  </si>
-  <si>
-    <t>ahmetyılmaz@gmail.com</t>
-  </si>
-  <si>
     <t>aysedemir@gmail.com</t>
   </si>
   <si>
-    <t>Varoloooo</t>
+    <t>05551112233</t>
+  </si>
+  <si>
+    <t>Varol</t>
   </si>
 </sst>
 </file>
@@ -90,7 +93,6 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
@@ -117,16 +119,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Köprü" xfId="1" builtinId="8"/>
+    <cellStyle name="Köprü" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -139,7 +142,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -181,74 +184,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -256,55 +199,15 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="dk1"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="accent1"/>
+        </a:solidFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -313,13 +216,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -353,24 +256,13 @@
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -396,7 +288,7 @@
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -434,34 +326,34 @@
     <col min="4" max="4" width="16.85546875" customWidth="1"/>
     <col min="5" max="5" width="17.85546875" customWidth="1"/>
     <col min="6" max="6" width="16.5703125" customWidth="1"/>
-    <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17" customWidth="1"/>
     <col min="8" max="8" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" t="s">
-        <v>4</v>
-      </c>
       <c r="H1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -469,19 +361,19 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2">
-        <v>5551112233</v>
-      </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -495,19 +387,19 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3">
-        <v>5551112233</v>
+        <v>13</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>18</v>
       </c>
       <c r="F3" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -521,19 +413,19 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E4">
-        <v>5551112233</v>
+      <c r="E4" s="2" t="s">
+        <v>18</v>
       </c>
       <c r="F4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G4">
         <v>1</v>
@@ -543,11 +435,6 @@
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" xr:uid="{9C469817-3926-4F8D-B5ED-8556D44BDE9B}"/>
-    <hyperlink ref="D3" r:id="rId2" xr:uid="{3690221B-13B7-46CD-97F5-2E6760F937F2}"/>
-    <hyperlink ref="D4" r:id="rId3" xr:uid="{799CCEB2-4032-4FB2-AD04-A24C627D1575}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add styling to butons for smaller font size
</commit_message>
<xml_diff>
--- a/wwwroot/templates/KullaniciTemplate.xlsx
+++ b/wwwroot/templates/KullaniciTemplate.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOD\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EMutabakat\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F117C2D-5886-420E-8AA7-B670E00F72D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2025D933-4DBC-49D5-8DCB-E140FF06EFB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="690" yWindow="4275" windowWidth="16950" windowHeight="10950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2580" yWindow="4350" windowWidth="16950" windowHeight="10950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="21">
   <si>
     <t>KullaniciId</t>
   </si>
@@ -80,6 +80,9 @@
   </si>
   <si>
     <t>Varol</t>
+  </si>
+  <si>
+    <t>05554444444</t>
   </si>
 </sst>
 </file>
@@ -370,7 +373,7 @@
         <v>9</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F2" t="s">
         <v>10</v>

</xml_diff>